<commit_message>
chore: add description for xlsx template
</commit_message>
<xml_diff>
--- a/cypress/downloads/modele_sms_destinataires.xlsx
+++ b/cypress/downloads/modele_sms_destinataires.xlsx
@@ -397,19 +397,31 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B1"/>
+  <dimension ref="A1:B2"/>
+  <cols>
+    <col min="1" max="1" width="40.83203125" customWidth="1"/>
+    <col min="2" max="2" width="60.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>Le message est optionnel si vous envoyez le même message à tous les destinataires : dans ce cas, laissez la colonne Message vide et utilisez le champ Message de l'interface web. Le message est obligatoire si vous voulez un message différent pour chaque destinataire.</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
         <v>Destinataire</v>
       </c>
-      <c r="B1" t="str">
-        <v>Message (optionnel)</v>
+      <c r="B2" t="str">
+        <v>Message</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B2"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>